<commit_message>
Rebuild Climbing Gym tab: fingerboard-first
Protocol-based logging matching Jo's training sheet: exercise presets, per-set loads with done-dots, both rests, RPE, auto Day Max / % of last max / %BM. Progress = Day Max trend + PBs. Old sessions preserved but hidden (fresh start)
</commit_message>
<xml_diff>
--- a/My Lattice&Climbing training docs/Jo_training raw docs 25_2026/myGym Training 25_2026.xlsx
+++ b/My Lattice&Climbing training docs/Jo_training raw docs 25_2026/myGym Training 25_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josinabernardes/Library/Mobile Documents/com~apple~CloudDocs/01 Claude in Docs/Jo files/Jo_training raw docs 25_2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josinabernardes/Documents/Tennis-Tracker-Hub/My Lattice&amp;Climbing training docs/Jo_training raw docs 25_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4153C2F7-24E3-C646-8844-EAAAE86246A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46E4923-42DC-964C-994E-64072AECA6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="15820" tabRatio="765" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="15820" tabRatio="765" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FH_25 Rehab" sheetId="6" r:id="rId1"/>
@@ -1548,7 +1548,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4692" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4692" uniqueCount="505">
   <si>
     <t>Training Gym 2024</t>
   </si>
@@ -3196,6 +3196,18 @@
   </si>
   <si>
     <t>Base 6c</t>
+  </si>
+  <si>
+    <t>Finger Borda</t>
+  </si>
+  <si>
+    <t>Fingers - Holds</t>
+  </si>
+  <si>
+    <t>Fingers - holds</t>
+  </si>
+  <si>
+    <t>Fingers -  holds</t>
   </si>
 </sst>
 </file>
@@ -5190,6 +5202,27 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -5205,38 +5238,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5256,14 +5265,17 @@
     <xf numFmtId="0" fontId="0" fillId="21" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -10982,17 +10994,17 @@
       <c r="I56" s="5"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="C59" s="393" t="s">
+      <c r="C59" s="388" t="s">
         <v>448</v>
       </c>
-      <c r="D59" s="393"/>
-      <c r="E59" s="393"/>
-      <c r="F59" s="393"/>
-      <c r="G59" s="393"/>
-      <c r="H59" s="393"/>
-      <c r="I59" s="393"/>
-      <c r="J59" s="393"/>
-      <c r="K59" s="393"/>
+      <c r="D59" s="388"/>
+      <c r="E59" s="388"/>
+      <c r="F59" s="388"/>
+      <c r="G59" s="388"/>
+      <c r="H59" s="388"/>
+      <c r="I59" s="388"/>
+      <c r="J59" s="388"/>
+      <c r="K59" s="388"/>
       <c r="M59" s="15" t="s">
         <v>429</v>
       </c>
@@ -12315,10 +12327,10 @@
       <c r="BV2" s="108" t="s">
         <v>36</v>
       </c>
-      <c r="CB2" s="385" t="s">
+      <c r="CB2" s="392" t="s">
         <v>482</v>
       </c>
-      <c r="CC2" s="386"/>
+      <c r="CC2" s="393"/>
       <c r="CD2" s="266">
         <v>2026</v>
       </c>
@@ -14054,13 +14066,13 @@
         <f>AE18*0.85</f>
         <v>25.074999999999999</v>
       </c>
-      <c r="CH18" s="389" t="s">
+      <c r="CH18" s="382" t="s">
         <v>397</v>
       </c>
-      <c r="CI18" s="387" t="s">
+      <c r="CI18" s="384" t="s">
         <v>492</v>
       </c>
-      <c r="CJ18" s="388"/>
+      <c r="CJ18" s="385"/>
     </row>
     <row r="19" spans="1:88" x14ac:dyDescent="0.2">
       <c r="A19">
@@ -14201,7 +14213,7 @@
       <c r="BZ19" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="CH19" s="390"/>
+      <c r="CH19" s="383"/>
       <c r="CI19" s="42" t="s">
         <v>398</v>
       </c>
@@ -14357,13 +14369,13 @@
       <c r="BZ20" s="45">
         <v>29.5</v>
       </c>
-      <c r="CH20" s="391" t="s">
+      <c r="CH20" s="386" t="s">
         <v>399</v>
       </c>
-      <c r="CI20" s="387" t="s">
+      <c r="CI20" s="384" t="s">
         <v>493</v>
       </c>
-      <c r="CJ20" s="388"/>
+      <c r="CJ20" s="385"/>
     </row>
     <row r="21" spans="1:88" x14ac:dyDescent="0.2">
       <c r="A21">
@@ -14505,7 +14517,7 @@
       <c r="BZ21" s="45">
         <v>16</v>
       </c>
-      <c r="CH21" s="392"/>
+      <c r="CH21" s="387"/>
       <c r="CI21" s="42" t="s">
         <v>398</v>
       </c>
@@ -19160,7 +19172,7 @@
         <v>1</v>
       </c>
       <c r="BS67" s="134" t="s">
-        <v>8</v>
+        <v>501</v>
       </c>
       <c r="BT67" s="126" t="s">
         <v>14</v>
@@ -20232,7 +20244,7 @@
         <v>2</v>
       </c>
       <c r="BS82" s="134" t="s">
-        <v>8</v>
+        <v>502</v>
       </c>
       <c r="BT82" s="126" t="s">
         <v>14</v>
@@ -20485,7 +20497,7 @@
         <v>3</v>
       </c>
       <c r="BS85" s="134" t="s">
-        <v>8</v>
+        <v>503</v>
       </c>
       <c r="BT85" s="126" t="s">
         <v>14</v>
@@ -20738,7 +20750,7 @@
         <v>4</v>
       </c>
       <c r="BS88" s="134" t="s">
-        <v>8</v>
+        <v>503</v>
       </c>
       <c r="BT88" s="126" t="s">
         <v>14</v>
@@ -20991,7 +21003,7 @@
         <v>5</v>
       </c>
       <c r="BS91" s="134" t="s">
-        <v>8</v>
+        <v>504</v>
       </c>
       <c r="BT91" s="126" t="s">
         <v>14</v>
@@ -27032,7 +27044,7 @@
     <row r="169" spans="35:81" ht="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="172" spans="35:81" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="173" spans="35:81" x14ac:dyDescent="0.2">
-      <c r="AI173" s="382" t="s">
+      <c r="AI173" s="389" t="s">
         <v>241</v>
       </c>
       <c r="AJ173" s="151" t="s">
@@ -27068,7 +27080,7 @@
       <c r="AT173" s="51" t="s">
         <v>235</v>
       </c>
-      <c r="BA173" s="382" t="s">
+      <c r="BA173" s="389" t="s">
         <v>241</v>
       </c>
       <c r="BB173" s="151" t="s">
@@ -27104,7 +27116,7 @@
       <c r="BL173" s="51" t="s">
         <v>235</v>
       </c>
-      <c r="BR173" s="382" t="s">
+      <c r="BR173" s="389" t="s">
         <v>241</v>
       </c>
       <c r="BS173" s="151" t="s">
@@ -27142,7 +27154,7 @@
       </c>
     </row>
     <row r="174" spans="35:81" x14ac:dyDescent="0.2">
-      <c r="AI174" s="383"/>
+      <c r="AI174" s="390"/>
       <c r="AJ174" s="39" t="s">
         <v>240</v>
       </c>
@@ -27176,7 +27188,7 @@
       <c r="AT174" s="53" t="s">
         <v>236</v>
       </c>
-      <c r="BA174" s="383"/>
+      <c r="BA174" s="390"/>
       <c r="BB174" s="39" t="s">
         <v>240</v>
       </c>
@@ -27210,7 +27222,7 @@
       <c r="BL174" s="53" t="s">
         <v>236</v>
       </c>
-      <c r="BR174" s="383"/>
+      <c r="BR174" s="390"/>
       <c r="BS174" s="39" t="s">
         <v>240</v>
       </c>
@@ -27246,15 +27258,15 @@
       </c>
     </row>
     <row r="175" spans="35:81" x14ac:dyDescent="0.2">
-      <c r="AI175" s="383"/>
+      <c r="AI175" s="390"/>
       <c r="AT175" s="155"/>
-      <c r="BA175" s="383"/>
+      <c r="BA175" s="390"/>
       <c r="BL175" s="155"/>
-      <c r="BR175" s="383"/>
+      <c r="BR175" s="390"/>
       <c r="CC175" s="155"/>
     </row>
     <row r="176" spans="35:81" x14ac:dyDescent="0.2">
-      <c r="AI176" s="383"/>
+      <c r="AI176" s="390"/>
       <c r="AJ176" s="136" t="s">
         <v>234</v>
       </c>
@@ -27288,7 +27300,7 @@
       <c r="AT176" s="53" t="s">
         <v>235</v>
       </c>
-      <c r="BA176" s="383"/>
+      <c r="BA176" s="390"/>
       <c r="BB176" s="136" t="s">
         <v>234</v>
       </c>
@@ -27322,7 +27334,7 @@
       <c r="BL176" s="53" t="s">
         <v>235</v>
       </c>
-      <c r="BR176" s="383"/>
+      <c r="BR176" s="390"/>
       <c r="BS176" s="136" t="s">
         <v>234</v>
       </c>
@@ -27358,7 +27370,7 @@
       </c>
     </row>
     <row r="177" spans="35:81" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="AI177" s="384"/>
+      <c r="AI177" s="391"/>
       <c r="AJ177" s="156" t="s">
         <v>239</v>
       </c>
@@ -27392,7 +27404,7 @@
       <c r="AT177" s="43" t="s">
         <v>242</v>
       </c>
-      <c r="BA177" s="384"/>
+      <c r="BA177" s="391"/>
       <c r="BB177" s="156" t="s">
         <v>239</v>
       </c>
@@ -27426,7 +27438,7 @@
       <c r="BL177" s="43" t="s">
         <v>242</v>
       </c>
-      <c r="BR177" s="384"/>
+      <c r="BR177" s="391"/>
       <c r="BS177" s="156" t="s">
         <v>239</v>
       </c>
@@ -28803,32 +28815,32 @@
       <c r="F16" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="389" t="s">
+      <c r="A18" s="382" t="s">
         <v>397</v>
       </c>
-      <c r="B18" s="387" t="s">
+      <c r="B18" s="384" t="s">
         <v>492</v>
       </c>
-      <c r="C18" s="388"/>
+      <c r="C18" s="385"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="390"/>
+      <c r="A19" s="383"/>
       <c r="B19" s="42" t="s">
         <v>398</v>
       </c>
       <c r="C19" s="42"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="391" t="s">
+      <c r="A20" s="386" t="s">
         <v>399</v>
       </c>
-      <c r="B20" s="387" t="s">
+      <c r="B20" s="384" t="s">
         <v>493</v>
       </c>
-      <c r="C20" s="388"/>
+      <c r="C20" s="385"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="392"/>
+      <c r="A21" s="387"/>
       <c r="B21" s="42" t="s">
         <v>398</v>
       </c>
@@ -29150,36 +29162,36 @@
     </row>
     <row r="24" spans="1:31" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:31" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="401"/>
-      <c r="C25" s="402"/>
-      <c r="D25" s="402"/>
-      <c r="E25" s="402"/>
-      <c r="F25" s="402"/>
-      <c r="G25" s="402"/>
-      <c r="H25" s="402"/>
-      <c r="I25" s="402"/>
-      <c r="J25" s="402"/>
-      <c r="K25" s="402"/>
-      <c r="L25" s="402"/>
-      <c r="M25" s="402"/>
-      <c r="N25" s="402"/>
-      <c r="O25" s="402"/>
-      <c r="P25" s="402"/>
-      <c r="Q25" s="402"/>
-      <c r="R25" s="402"/>
-      <c r="S25" s="402"/>
-      <c r="T25" s="402"/>
-      <c r="U25" s="402"/>
-      <c r="V25" s="402"/>
-      <c r="W25" s="402"/>
-      <c r="X25" s="402"/>
-      <c r="Y25" s="402"/>
-      <c r="Z25" s="402"/>
-      <c r="AA25" s="402"/>
-      <c r="AB25" s="402"/>
-      <c r="AC25" s="402"/>
-      <c r="AD25" s="402"/>
-      <c r="AE25" s="403"/>
+      <c r="B25" s="400"/>
+      <c r="C25" s="401"/>
+      <c r="D25" s="401"/>
+      <c r="E25" s="401"/>
+      <c r="F25" s="401"/>
+      <c r="G25" s="401"/>
+      <c r="H25" s="401"/>
+      <c r="I25" s="401"/>
+      <c r="J25" s="401"/>
+      <c r="K25" s="401"/>
+      <c r="L25" s="401"/>
+      <c r="M25" s="401"/>
+      <c r="N25" s="401"/>
+      <c r="O25" s="401"/>
+      <c r="P25" s="401"/>
+      <c r="Q25" s="401"/>
+      <c r="R25" s="401"/>
+      <c r="S25" s="401"/>
+      <c r="T25" s="401"/>
+      <c r="U25" s="401"/>
+      <c r="V25" s="401"/>
+      <c r="W25" s="401"/>
+      <c r="X25" s="401"/>
+      <c r="Y25" s="401"/>
+      <c r="Z25" s="401"/>
+      <c r="AA25" s="401"/>
+      <c r="AB25" s="401"/>
+      <c r="AC25" s="401"/>
+      <c r="AD25" s="401"/>
+      <c r="AE25" s="402"/>
     </row>
     <row r="28" spans="1:31" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="L28" s="18" t="s">
@@ -29263,79 +29275,79 @@
       </c>
     </row>
     <row r="35" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N35" s="398" t="s">
+      <c r="N35" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="O35" s="399"/>
-      <c r="P35" s="399"/>
-      <c r="Q35" s="400"/>
-      <c r="S35" s="398" t="s">
+      <c r="O35" s="398"/>
+      <c r="P35" s="398"/>
+      <c r="Q35" s="399"/>
+      <c r="S35" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="T35" s="399"/>
-      <c r="U35" s="399"/>
-      <c r="V35" s="400"/>
-      <c r="X35" s="398" t="s">
+      <c r="T35" s="398"/>
+      <c r="U35" s="398"/>
+      <c r="V35" s="399"/>
+      <c r="X35" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="Y35" s="399"/>
-      <c r="Z35" s="399"/>
-      <c r="AA35" s="400"/>
-      <c r="AC35" s="398" t="s">
+      <c r="Y35" s="398"/>
+      <c r="Z35" s="398"/>
+      <c r="AA35" s="399"/>
+      <c r="AC35" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="AD35" s="399"/>
-      <c r="AE35" s="399"/>
-      <c r="AF35" s="400"/>
-      <c r="AH35" s="398" t="s">
+      <c r="AD35" s="398"/>
+      <c r="AE35" s="398"/>
+      <c r="AF35" s="399"/>
+      <c r="AH35" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="AI35" s="399"/>
-      <c r="AJ35" s="399"/>
-      <c r="AK35" s="400"/>
+      <c r="AI35" s="398"/>
+      <c r="AJ35" s="398"/>
+      <c r="AK35" s="399"/>
     </row>
     <row r="36" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N36" s="398">
+      <c r="N36" s="397">
         <v>1</v>
       </c>
-      <c r="O36" s="399"/>
-      <c r="P36" s="399"/>
+      <c r="O36" s="398"/>
+      <c r="P36" s="398"/>
       <c r="Q36" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="S36" s="398">
+      <c r="S36" s="397">
         <f>N36+1</f>
         <v>2</v>
       </c>
-      <c r="T36" s="399"/>
-      <c r="U36" s="399"/>
+      <c r="T36" s="398"/>
+      <c r="U36" s="398"/>
       <c r="V36" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="X36" s="398">
+      <c r="X36" s="397">
         <f>S36+1</f>
         <v>3</v>
       </c>
-      <c r="Y36" s="399"/>
-      <c r="Z36" s="399"/>
+      <c r="Y36" s="398"/>
+      <c r="Z36" s="398"/>
       <c r="AA36" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="AC36" s="398">
+      <c r="AC36" s="397">
         <f>X36+1</f>
         <v>4</v>
       </c>
-      <c r="AD36" s="399"/>
-      <c r="AE36" s="399"/>
+      <c r="AD36" s="398"/>
+      <c r="AE36" s="398"/>
       <c r="AF36" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="AH36" s="398">
+      <c r="AH36" s="397">
         <f>AC36+1</f>
         <v>5</v>
       </c>
-      <c r="AI36" s="399"/>
-      <c r="AJ36" s="399"/>
+      <c r="AI36" s="398"/>
+      <c r="AJ36" s="398"/>
       <c r="AK36" s="319" t="s">
         <v>148</v>
       </c>
@@ -30745,35 +30757,35 @@
       <c r="M55" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="N55" s="404"/>
-      <c r="O55" s="405"/>
-      <c r="P55" s="406"/>
+      <c r="N55" s="394"/>
+      <c r="O55" s="395"/>
+      <c r="P55" s="396"/>
       <c r="R55" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="S55" s="404" t="s">
+      <c r="S55" s="394" t="s">
         <v>494</v>
       </c>
-      <c r="T55" s="405"/>
-      <c r="U55" s="406"/>
+      <c r="T55" s="395"/>
+      <c r="U55" s="396"/>
       <c r="W55" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="X55" s="404"/>
-      <c r="Y55" s="405"/>
-      <c r="Z55" s="406"/>
+      <c r="X55" s="394"/>
+      <c r="Y55" s="395"/>
+      <c r="Z55" s="396"/>
       <c r="AB55" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="AC55" s="404"/>
-      <c r="AD55" s="405"/>
-      <c r="AE55" s="406"/>
+      <c r="AC55" s="394"/>
+      <c r="AD55" s="395"/>
+      <c r="AE55" s="396"/>
       <c r="AG55" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="AH55" s="404"/>
-      <c r="AI55" s="405"/>
-      <c r="AJ55" s="406"/>
+      <c r="AH55" s="394"/>
+      <c r="AI55" s="395"/>
+      <c r="AJ55" s="396"/>
     </row>
     <row r="56" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B56" s="377" t="s">
@@ -31046,10 +31058,10 @@
       </c>
     </row>
     <row r="70" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="L70" s="394" t="s">
+      <c r="L70" s="403" t="s">
         <v>473</v>
       </c>
-      <c r="M70" s="395"/>
+      <c r="M70" s="404"/>
       <c r="N70" s="122">
         <f>Q39+V39+AA39+AF39+AK39</f>
         <v>1157</v>
@@ -31064,10 +31076,10 @@
       </c>
     </row>
     <row r="71" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="L71" s="396" t="s">
+      <c r="L71" s="405" t="s">
         <v>474</v>
       </c>
-      <c r="M71" s="397"/>
+      <c r="M71" s="406"/>
       <c r="N71" s="302"/>
       <c r="O71" s="302"/>
       <c r="P71" s="298">
@@ -31076,10 +31088,10 @@
       </c>
     </row>
     <row r="72" spans="2:31" x14ac:dyDescent="0.2">
-      <c r="L72" s="396" t="s">
+      <c r="L72" s="405" t="s">
         <v>475</v>
       </c>
-      <c r="M72" s="397"/>
+      <c r="M72" s="406"/>
       <c r="N72" s="302"/>
       <c r="O72" s="302"/>
       <c r="P72" s="298">
@@ -31089,36 +31101,36 @@
     </row>
     <row r="74" spans="2:31" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="75" spans="2:31" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="401"/>
-      <c r="C75" s="402"/>
-      <c r="D75" s="402"/>
-      <c r="E75" s="402"/>
-      <c r="F75" s="402"/>
-      <c r="G75" s="402"/>
-      <c r="H75" s="402"/>
-      <c r="I75" s="402"/>
-      <c r="J75" s="402"/>
-      <c r="K75" s="402"/>
-      <c r="L75" s="402"/>
-      <c r="M75" s="402"/>
-      <c r="N75" s="402"/>
-      <c r="O75" s="402"/>
-      <c r="P75" s="402"/>
-      <c r="Q75" s="402"/>
-      <c r="R75" s="402"/>
-      <c r="S75" s="402"/>
-      <c r="T75" s="402"/>
-      <c r="U75" s="402"/>
-      <c r="V75" s="402"/>
-      <c r="W75" s="402"/>
-      <c r="X75" s="402"/>
-      <c r="Y75" s="402"/>
-      <c r="Z75" s="402"/>
-      <c r="AA75" s="402"/>
-      <c r="AB75" s="402"/>
-      <c r="AC75" s="402"/>
-      <c r="AD75" s="402"/>
-      <c r="AE75" s="403"/>
+      <c r="B75" s="400"/>
+      <c r="C75" s="401"/>
+      <c r="D75" s="401"/>
+      <c r="E75" s="401"/>
+      <c r="F75" s="401"/>
+      <c r="G75" s="401"/>
+      <c r="H75" s="401"/>
+      <c r="I75" s="401"/>
+      <c r="J75" s="401"/>
+      <c r="K75" s="401"/>
+      <c r="L75" s="401"/>
+      <c r="M75" s="401"/>
+      <c r="N75" s="401"/>
+      <c r="O75" s="401"/>
+      <c r="P75" s="401"/>
+      <c r="Q75" s="401"/>
+      <c r="R75" s="401"/>
+      <c r="S75" s="401"/>
+      <c r="T75" s="401"/>
+      <c r="U75" s="401"/>
+      <c r="V75" s="401"/>
+      <c r="W75" s="401"/>
+      <c r="X75" s="401"/>
+      <c r="Y75" s="401"/>
+      <c r="Z75" s="401"/>
+      <c r="AA75" s="401"/>
+      <c r="AB75" s="401"/>
+      <c r="AC75" s="401"/>
+      <c r="AD75" s="401"/>
+      <c r="AE75" s="402"/>
     </row>
     <row r="78" spans="2:31" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="L78" s="18" t="s">
@@ -31192,79 +31204,79 @@
       </c>
     </row>
     <row r="85" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N85" s="398" t="s">
+      <c r="N85" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="O85" s="399"/>
-      <c r="P85" s="399"/>
-      <c r="Q85" s="400"/>
-      <c r="S85" s="398" t="s">
+      <c r="O85" s="398"/>
+      <c r="P85" s="398"/>
+      <c r="Q85" s="399"/>
+      <c r="S85" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="T85" s="399"/>
-      <c r="U85" s="399"/>
-      <c r="V85" s="400"/>
-      <c r="X85" s="398" t="s">
+      <c r="T85" s="398"/>
+      <c r="U85" s="398"/>
+      <c r="V85" s="399"/>
+      <c r="X85" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="Y85" s="399"/>
-      <c r="Z85" s="399"/>
-      <c r="AA85" s="400"/>
-      <c r="AC85" s="398" t="s">
+      <c r="Y85" s="398"/>
+      <c r="Z85" s="398"/>
+      <c r="AA85" s="399"/>
+      <c r="AC85" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="AD85" s="399"/>
-      <c r="AE85" s="399"/>
-      <c r="AF85" s="400"/>
-      <c r="AH85" s="398" t="s">
+      <c r="AD85" s="398"/>
+      <c r="AE85" s="398"/>
+      <c r="AF85" s="399"/>
+      <c r="AH85" s="397" t="s">
         <v>136</v>
       </c>
-      <c r="AI85" s="399"/>
-      <c r="AJ85" s="399"/>
-      <c r="AK85" s="400"/>
+      <c r="AI85" s="398"/>
+      <c r="AJ85" s="398"/>
+      <c r="AK85" s="399"/>
     </row>
     <row r="86" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="N86" s="398">
+      <c r="N86" s="397">
         <v>5</v>
       </c>
-      <c r="O86" s="399"/>
-      <c r="P86" s="399"/>
+      <c r="O86" s="398"/>
+      <c r="P86" s="398"/>
       <c r="Q86" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="S86" s="398">
+      <c r="S86" s="397">
         <f>N86+1</f>
         <v>6</v>
       </c>
-      <c r="T86" s="399"/>
-      <c r="U86" s="399"/>
+      <c r="T86" s="398"/>
+      <c r="U86" s="398"/>
       <c r="V86" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="X86" s="398">
+      <c r="X86" s="397">
         <f>S86+1</f>
         <v>7</v>
       </c>
-      <c r="Y86" s="399"/>
-      <c r="Z86" s="399"/>
+      <c r="Y86" s="398"/>
+      <c r="Z86" s="398"/>
       <c r="AA86" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="AC86" s="398">
+      <c r="AC86" s="397">
         <f>X86+1</f>
         <v>8</v>
       </c>
-      <c r="AD86" s="399"/>
-      <c r="AE86" s="399"/>
+      <c r="AD86" s="398"/>
+      <c r="AE86" s="398"/>
       <c r="AF86" s="319" t="s">
         <v>148</v>
       </c>
-      <c r="AH86" s="398">
+      <c r="AH86" s="397">
         <f>AC86+1</f>
         <v>9</v>
       </c>
-      <c r="AI86" s="399"/>
-      <c r="AJ86" s="399"/>
+      <c r="AI86" s="398"/>
+      <c r="AJ86" s="398"/>
       <c r="AK86" s="319" t="s">
         <v>148</v>
       </c>
@@ -32506,33 +32518,33 @@
       <c r="M105" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="N105" s="404"/>
-      <c r="O105" s="405"/>
-      <c r="P105" s="406"/>
+      <c r="N105" s="394"/>
+      <c r="O105" s="395"/>
+      <c r="P105" s="396"/>
       <c r="R105" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="S105" s="404"/>
-      <c r="T105" s="405"/>
-      <c r="U105" s="406"/>
+      <c r="S105" s="394"/>
+      <c r="T105" s="395"/>
+      <c r="U105" s="396"/>
       <c r="W105" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="X105" s="404"/>
-      <c r="Y105" s="405"/>
-      <c r="Z105" s="406"/>
+      <c r="X105" s="394"/>
+      <c r="Y105" s="395"/>
+      <c r="Z105" s="396"/>
       <c r="AB105" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="AC105" s="404"/>
-      <c r="AD105" s="405"/>
-      <c r="AE105" s="406"/>
+      <c r="AC105" s="394"/>
+      <c r="AD105" s="395"/>
+      <c r="AE105" s="396"/>
       <c r="AG105" s="115" t="s">
         <v>217</v>
       </c>
-      <c r="AH105" s="404"/>
-      <c r="AI105" s="405"/>
-      <c r="AJ105" s="406"/>
+      <c r="AH105" s="394"/>
+      <c r="AI105" s="395"/>
+      <c r="AJ105" s="396"/>
     </row>
     <row r="106" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="107" spans="2:37" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -32673,10 +32685,10 @@
       </c>
     </row>
     <row r="120" spans="12:16" x14ac:dyDescent="0.2">
-      <c r="L120" s="394" t="s">
+      <c r="L120" s="403" t="s">
         <v>473</v>
       </c>
-      <c r="M120" s="395"/>
+      <c r="M120" s="404"/>
       <c r="N120" s="122">
         <f>Q89+V89+AA89+AF89+AK89</f>
         <v>0</v>
@@ -32691,10 +32703,10 @@
       </c>
     </row>
     <row r="121" spans="12:16" x14ac:dyDescent="0.2">
-      <c r="L121" s="396" t="s">
+      <c r="L121" s="405" t="s">
         <v>474</v>
       </c>
-      <c r="M121" s="397"/>
+      <c r="M121" s="406"/>
       <c r="N121" s="302"/>
       <c r="O121" s="302"/>
       <c r="P121" s="298">
@@ -32703,10 +32715,10 @@
       </c>
     </row>
     <row r="122" spans="12:16" x14ac:dyDescent="0.2">
-      <c r="L122" s="396" t="s">
+      <c r="L122" s="405" t="s">
         <v>475</v>
       </c>
-      <c r="M122" s="397"/>
+      <c r="M122" s="406"/>
       <c r="N122" s="302"/>
       <c r="O122" s="302"/>
       <c r="P122" s="298">
@@ -32716,21 +32728,17 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="AH55:AJ55"/>
-    <mergeCell ref="N105:P105"/>
-    <mergeCell ref="S105:U105"/>
-    <mergeCell ref="X105:Z105"/>
-    <mergeCell ref="AC105:AE105"/>
-    <mergeCell ref="AH105:AJ105"/>
-    <mergeCell ref="AH86:AJ86"/>
-    <mergeCell ref="AH85:AK85"/>
-    <mergeCell ref="B25:AE25"/>
-    <mergeCell ref="S55:U55"/>
-    <mergeCell ref="N55:P55"/>
-    <mergeCell ref="X55:Z55"/>
-    <mergeCell ref="AC55:AE55"/>
-    <mergeCell ref="X36:Z36"/>
-    <mergeCell ref="AC36:AE36"/>
+    <mergeCell ref="L70:M70"/>
+    <mergeCell ref="L71:M71"/>
+    <mergeCell ref="L72:M72"/>
+    <mergeCell ref="N36:P36"/>
+    <mergeCell ref="S36:U36"/>
+    <mergeCell ref="AH36:AJ36"/>
+    <mergeCell ref="N35:Q35"/>
+    <mergeCell ref="S35:V35"/>
+    <mergeCell ref="X35:AA35"/>
+    <mergeCell ref="AC35:AF35"/>
+    <mergeCell ref="AH35:AK35"/>
     <mergeCell ref="L120:M120"/>
     <mergeCell ref="L121:M121"/>
     <mergeCell ref="L122:M122"/>
@@ -32743,17 +32751,21 @@
     <mergeCell ref="S85:V85"/>
     <mergeCell ref="X85:AA85"/>
     <mergeCell ref="AC85:AF85"/>
-    <mergeCell ref="AH36:AJ36"/>
-    <mergeCell ref="N35:Q35"/>
-    <mergeCell ref="S35:V35"/>
-    <mergeCell ref="X35:AA35"/>
-    <mergeCell ref="AC35:AF35"/>
-    <mergeCell ref="AH35:AK35"/>
-    <mergeCell ref="L70:M70"/>
-    <mergeCell ref="L71:M71"/>
-    <mergeCell ref="L72:M72"/>
-    <mergeCell ref="N36:P36"/>
-    <mergeCell ref="S36:U36"/>
+    <mergeCell ref="B25:AE25"/>
+    <mergeCell ref="S55:U55"/>
+    <mergeCell ref="N55:P55"/>
+    <mergeCell ref="X55:Z55"/>
+    <mergeCell ref="AC55:AE55"/>
+    <mergeCell ref="X36:Z36"/>
+    <mergeCell ref="AC36:AE36"/>
+    <mergeCell ref="AH55:AJ55"/>
+    <mergeCell ref="N105:P105"/>
+    <mergeCell ref="S105:U105"/>
+    <mergeCell ref="X105:Z105"/>
+    <mergeCell ref="AC105:AE105"/>
+    <mergeCell ref="AH105:AJ105"/>
+    <mergeCell ref="AH86:AJ86"/>
+    <mergeCell ref="AH85:AK85"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -33681,17 +33693,17 @@
       <c r="Z37" s="257" t="s">
         <v>411</v>
       </c>
-      <c r="AG37" s="398" t="s">
+      <c r="AG37" s="397" t="s">
         <v>203</v>
       </c>
-      <c r="AH37" s="399"/>
-      <c r="AI37" s="399"/>
-      <c r="AJ37" s="399"/>
-      <c r="AK37" s="399"/>
-      <c r="AL37" s="399"/>
-      <c r="AM37" s="399"/>
-      <c r="AN37" s="399"/>
-      <c r="AO37" s="400"/>
+      <c r="AH37" s="398"/>
+      <c r="AI37" s="398"/>
+      <c r="AJ37" s="398"/>
+      <c r="AK37" s="398"/>
+      <c r="AL37" s="398"/>
+      <c r="AM37" s="398"/>
+      <c r="AN37" s="398"/>
+      <c r="AO37" s="399"/>
     </row>
     <row r="38" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="407" t="s">
@@ -33738,11 +33750,11 @@
         <v>362</v>
       </c>
       <c r="O39" s="411"/>
-      <c r="P39" s="398" t="s">
+      <c r="P39" s="397" t="s">
         <v>449</v>
       </c>
-      <c r="Q39" s="399"/>
-      <c r="R39" s="400"/>
+      <c r="Q39" s="398"/>
+      <c r="R39" s="399"/>
       <c r="W39" s="412" t="s">
         <v>412</v>
       </c>

</xml_diff>